<commit_message>
refactor: update question generation and assessment schemas for BFI2
- Modified question generation scripts to enhance prompt formatting for BFI2 assessments.
- Updated assessment session schema to include assessment type, improving session tracking.
- Enhanced assessment routes to support new assessment type handling and history retrieval functionality.
</commit_message>
<xml_diff>
--- a/scripts/questions_test.xlsx
+++ b/scripts/questions_test.xlsx
@@ -449,7 +449,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>我是一个……的人 1. 性格外向，喜欢交际</v>
+        <v>我是一个性格外向，喜欢交际的人</v>
       </c>
       <c r="B2" t="str">
         <v>BIG5</v>
@@ -484,7 +484,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>我是一个……的人 2. 心肠柔软，有同情心</v>
+        <v>我是一个心肠柔软，有同情心的人</v>
       </c>
       <c r="B3" t="str">
         <v>BIG5</v>
@@ -519,7 +519,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>我是一个……的人 3. 缺乏条理</v>
+        <v>我是一个缺乏条理的人</v>
       </c>
       <c r="B4" t="str">
         <v>BIG5</v>
@@ -554,7 +554,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>我是一个……的人 4. 从容，善于处理压力</v>
+        <v>我是一个从容，善于处理压力的人</v>
       </c>
       <c r="B5" t="str">
         <v>BIG5</v>
@@ -589,7 +589,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>我是一个……的人 5. 对艺术没有什么兴趣</v>
+        <v>我是一个对艺术没有什么兴趣的人</v>
       </c>
       <c r="B6" t="str">
         <v>BIG5</v>
@@ -624,7 +624,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>我是一个……的人 6. 性格坚定自信，敢于表达自己的观点</v>
+        <v>我是一个性格坚定自信，敢于表达自己的观点的人</v>
       </c>
       <c r="B7" t="str">
         <v>BIG5</v>
@@ -659,7 +659,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>我是一个……的人 7. 为人恭谦，尊重他人</v>
+        <v>我是一个为人恭谦，尊重他人的人</v>
       </c>
       <c r="B8" t="str">
         <v>BIG5</v>
@@ -694,7 +694,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>我是一个……的人 8. 比较懒</v>
+        <v>我是一个比较懒的人</v>
       </c>
       <c r="B9" t="str">
         <v>BIG5</v>
@@ -729,7 +729,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>我是一个……的人 9. 经历挫折后仍能保持积极心态</v>
+        <v>我是一个经历挫折后仍能保持积极心态的人</v>
       </c>
       <c r="B10" t="str">
         <v>BIG5</v>
@@ -764,7 +764,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>我是一个……的人 10. 对许多不同的事物都感兴趣</v>
+        <v>我是一个对许多不同的事物都感兴趣的人</v>
       </c>
       <c r="B11" t="str">
         <v>BIG5</v>
@@ -799,7 +799,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>我是一个……的人 11. 很少觉得兴奋或者特别想要(做)什么</v>
+        <v>我是一个很少觉得兴奋或者特别想要(做)什么的人</v>
       </c>
       <c r="B12" t="str">
         <v>BIG5</v>
@@ -834,7 +834,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>我是一个……的人 12. 常常挑别人的毛病</v>
+        <v>我是一个常常挑别人的毛病的人</v>
       </c>
       <c r="B13" t="str">
         <v>BIG5</v>
@@ -869,7 +869,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>我是一个……的人 13. 可信赖的，可靠的</v>
+        <v>我是一个可信赖的，可靠的的人</v>
       </c>
       <c r="B14" t="str">
         <v>BIG5</v>
@@ -904,7 +904,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>我是一个……的人 14. 喜怒无常，情绪起伏较多</v>
+        <v>我是一个喜怒无常，情绪起伏较多的人</v>
       </c>
       <c r="B15" t="str">
         <v>BIG5</v>
@@ -939,7 +939,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>我是一个……的人 15. 善于创造，能找到聪明的方法来做事</v>
+        <v>我是一个善于创造，能找到聪明的方法来做事的人</v>
       </c>
       <c r="B16" t="str">
         <v>BIG5</v>
@@ -974,7 +974,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>我是一个……的人 16. 比较安静</v>
+        <v>我是一个比较安静的人</v>
       </c>
       <c r="B17" t="str">
         <v>BIG5</v>
@@ -1009,7 +1009,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>我是一个……的人 17. 对他人没有什么同情心</v>
+        <v>我是一个对他人没有什么同情心的人</v>
       </c>
       <c r="B18" t="str">
         <v>BIG5</v>
@@ -1044,7 +1044,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>我是一个……的人 18. 做事有计划有条理</v>
+        <v>我是一个做事有计划有条理的人</v>
       </c>
       <c r="B19" t="str">
         <v>BIG5</v>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>我是一个……的人 19. 容易紧张</v>
+        <v>我是一个容易紧张的人</v>
       </c>
       <c r="B20" t="str">
         <v>BIG5</v>
@@ -1114,7 +1114,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>我是一个……的人 20. 着迷于艺术、音乐或文学</v>
+        <v>我是一个着迷于艺术、音乐或文学的人</v>
       </c>
       <c r="B21" t="str">
         <v>BIG5</v>
@@ -1149,7 +1149,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>我是一个……的人 21. 常常处于主导地位，像个领导一样</v>
+        <v>我是一个常常处于主导地位，像个领导一样的人</v>
       </c>
       <c r="B22" t="str">
         <v>BIG5</v>
@@ -1184,7 +1184,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>我是一个……的人 22. 常与他人意见不和</v>
+        <v>我是一个常与他人意见不和的人</v>
       </c>
       <c r="B23" t="str">
         <v>BIG5</v>
@@ -1219,7 +1219,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>我是一个……的人 23. 很难开始行动起来去完成一项任务</v>
+        <v>我是一个很难开始行动起来去完成一项任务的人</v>
       </c>
       <c r="B24" t="str">
         <v>BIG5</v>
@@ -1254,7 +1254,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>我是一个……的人 24. 觉得有安全感，对自己满意</v>
+        <v>我是一个觉得有安全感，对自己满意的人</v>
       </c>
       <c r="B25" t="str">
         <v>BIG5</v>
@@ -1289,7 +1289,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>我是一个……的人 25. 不喜欢知识性或者哲学性强的讨论</v>
+        <v>我是一个不喜欢知识性或者哲学性强的讨论的人</v>
       </c>
       <c r="B26" t="str">
         <v>BIG5</v>
@@ -1324,7 +1324,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>我是一个……的人 26. 不如别人有活力</v>
+        <v>我是一个不如别人有活力的人</v>
       </c>
       <c r="B27" t="str">
         <v>BIG5</v>
@@ -1359,7 +1359,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>我是一个……的人 27. 宽宏大量</v>
+        <v>我是一个宽宏大量的人</v>
       </c>
       <c r="B28" t="str">
         <v>BIG5</v>
@@ -1394,7 +1394,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>我是一个……的人 28. 有时比较没有责任心</v>
+        <v>我是一个有时比较没有责任心的人</v>
       </c>
       <c r="B29" t="str">
         <v>BIG5</v>
@@ -1429,7 +1429,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>我是一个……的人 29. 情绪稳定，不易生气</v>
+        <v>我是一个情绪稳定，不易生气的人</v>
       </c>
       <c r="B30" t="str">
         <v>BIG5</v>
@@ -1464,7 +1464,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>我是一个……的人 30. 几乎没有什么创造性</v>
+        <v>我是一个几乎没有什么创造性的人</v>
       </c>
       <c r="B31" t="str">
         <v>BIG5</v>
@@ -1499,7 +1499,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>我是一个……的人 31. 有时会害羞，比较内向</v>
+        <v>我是一个有时会害羞，比较内向的人</v>
       </c>
       <c r="B32" t="str">
         <v>BIG5</v>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>我是一个……的人 32. 乐于助人，待人无私</v>
+        <v>我是一个乐于助人，待人无私的人</v>
       </c>
       <c r="B33" t="str">
         <v>BIG5</v>
@@ -1569,7 +1569,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>我是一个……的人 33. 习惯让事物保持整洁有序</v>
+        <v>我是一个习惯让事物保持整洁有序的人</v>
       </c>
       <c r="B34" t="str">
         <v>BIG5</v>
@@ -1604,7 +1604,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>我是一个……的人 34. 时常忧心忡忡，担心很多事情</v>
+        <v>我是一个时常忧心忡忡，担心很多事情的人</v>
       </c>
       <c r="B35" t="str">
         <v>BIG5</v>
@@ -1639,7 +1639,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>我是一个……的人 35. 重视艺术与审美</v>
+        <v>我是一个重视艺术与审美的人</v>
       </c>
       <c r="B36" t="str">
         <v>BIG5</v>
@@ -1674,7 +1674,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>我是一个……的人 36. 感觉自己很难对他人产生影响</v>
+        <v>我是一个感觉自己很难对他人产生影响的人</v>
       </c>
       <c r="B37" t="str">
         <v>BIG5</v>
@@ -1709,7 +1709,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>我是一个……的人 37. 有时对人比较粗鲁</v>
+        <v>我是一个有时对人比较粗鲁的人</v>
       </c>
       <c r="B38" t="str">
         <v>BIG5</v>
@@ -1744,7 +1744,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>我是一个……的人 38. 有效率，做事有始有终</v>
+        <v>我是一个有效率，做事有始有终的人</v>
       </c>
       <c r="B39" t="str">
         <v>BIG5</v>
@@ -1779,7 +1779,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>我是一个……的人 39. 时常觉得悲伤</v>
+        <v>我是一个时常觉得悲伤的人</v>
       </c>
       <c r="B40" t="str">
         <v>BIG5</v>
@@ -1814,7 +1814,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>我是一个……的人 40. 思想深刻</v>
+        <v>我是一个思想深刻的人</v>
       </c>
       <c r="B41" t="str">
         <v>BIG5</v>
@@ -1849,7 +1849,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>我是一个……的人 41. 精力充沛</v>
+        <v>我是一个精力充沛的人</v>
       </c>
       <c r="B42" t="str">
         <v>BIG5</v>
@@ -1884,7 +1884,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>我是一个……的人 42. 不相信别人，怀疑别人的意图</v>
+        <v>我是一个不相信别人，怀疑别人的意图的人</v>
       </c>
       <c r="B43" t="str">
         <v>BIG5</v>
@@ -1919,7 +1919,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>我是一个……的人 43. 可靠的，总是值得他人信赖</v>
+        <v>我是一个可靠的，总是值得他人信赖的人</v>
       </c>
       <c r="B44" t="str">
         <v>BIG5</v>
@@ -1954,7 +1954,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>我是一个……的人 44. 能够控制自己的情绪</v>
+        <v>我是一个能够控制自己的情绪的人</v>
       </c>
       <c r="B45" t="str">
         <v>BIG5</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>我是一个……的人 45. 缺乏想象力</v>
+        <v>我是一个缺乏想象力的人</v>
       </c>
       <c r="B46" t="str">
         <v>BIG5</v>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>我是一个……的人 46. 爱说话，健谈</v>
+        <v>我是一个爱说话，健谈的人</v>
       </c>
       <c r="B47" t="str">
         <v>BIG5</v>
@@ -2059,7 +2059,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>我是一个……的人 47. 有时对人冷淡，漠不关心</v>
+        <v>我是一个有时对人冷淡，漠不关心的人</v>
       </c>
       <c r="B48" t="str">
         <v>BIG5</v>
@@ -2094,7 +2094,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>我是一个……的人 48. 乱糟糟的，不爱收拾</v>
+        <v>我是一个乱糟糟的，不爱收拾的人</v>
       </c>
       <c r="B49" t="str">
         <v>BIG5</v>
@@ -2129,7 +2129,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>我是一个……的人 49. 很少觉得焦虑或者害怕</v>
+        <v>我是一个很少觉得焦虑或者害怕的人</v>
       </c>
       <c r="B50" t="str">
         <v>BIG5</v>
@@ -2164,7 +2164,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>我是一个……的人 50. 觉得诗歌、戏剧很无聊</v>
+        <v>我是一个觉得诗歌、戏剧很无聊的人</v>
       </c>
       <c r="B51" t="str">
         <v>BIG5</v>
@@ -2199,7 +2199,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>我是一个……的人 51. 更喜欢让别人来领头负责</v>
+        <v>我是一个更喜欢让别人来领头负责的人</v>
       </c>
       <c r="B52" t="str">
         <v>BIG5</v>
@@ -2234,7 +2234,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>我是一个……的人 52. 待人谦逊礼让</v>
+        <v>我是一个待人谦逊礼让的人</v>
       </c>
       <c r="B53" t="str">
         <v>BIG5</v>
@@ -2269,7 +2269,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>我是一个……的人 53. 有恒心，能坚持把事情做完</v>
+        <v>我是一个有恒心，能坚持把事情做完的人</v>
       </c>
       <c r="B54" t="str">
         <v>BIG5</v>
@@ -2304,7 +2304,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>我是一个……的人 54. 时常觉得郁郁寡欢</v>
+        <v>我是一个时常觉得郁郁寡欢的人</v>
       </c>
       <c r="B55" t="str">
         <v>BIG5</v>
@@ -2339,7 +2339,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>我是一个……的人 55. 对抽象的概念和想法没什么兴趣</v>
+        <v>我是一个对抽象的概念和想法没什么兴趣的人</v>
       </c>
       <c r="B56" t="str">
         <v>BIG5</v>
@@ -2374,7 +2374,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>我是一个……的人 56. 充满热情</v>
+        <v>我是一个充满热情的人</v>
       </c>
       <c r="B57" t="str">
         <v>BIG5</v>
@@ -2409,7 +2409,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>我是一个……的人 57. 把人往最好的方面想</v>
+        <v>我是一个把人往最好的方面想的人</v>
       </c>
       <c r="B58" t="str">
         <v>BIG5</v>
@@ -2444,7 +2444,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>我是一个……的人 58. 有时候会做出一些不负责任的行为</v>
+        <v>我是一个有时候会做出一些不负责任的行为的人</v>
       </c>
       <c r="B59" t="str">
         <v>BIG5</v>
@@ -2479,7 +2479,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>我是一个……的人 59. 情绪多变，容易愤怒</v>
+        <v>我是一个情绪多变，容易愤怒的人</v>
       </c>
       <c r="B60" t="str">
         <v>BIG5</v>
@@ -2514,7 +2514,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>我是一个……的人 60. 有创意，能想出新点子</v>
+        <v>我是一个有创意，能想出新点子的人</v>
       </c>
       <c r="B61" t="str">
         <v>BIG5</v>

</xml_diff>